<commit_message>
Rerun the main.py after added robot.txt
Rerun the main.py after added robot.txt
</commit_message>
<xml_diff>
--- a/output/price_comparison_2plus_shops.xlsx
+++ b/output/price_comparison_2plus_shops.xlsx
@@ -46,61 +46,61 @@
     <t>LEGO 75442 The Mandalorian’s N-1 Starfighter</t>
   </si>
   <si>
-    <t>LEGO Icons 10337 Lamborghini Countach 5000...</t>
+    <t>LEGO 42688 Horse Stable and Riding Academy</t>
   </si>
   <si>
     <t>LEGO Friends 42673 Family Vacation Beach Resort...</t>
   </si>
   <si>
+    <t>LEGO 42689 Heartlake City Friends Club House</t>
+  </si>
+  <si>
     <t>LEGO City 60502 Airport with Airplane 60502</t>
   </si>
   <si>
+    <t>LEGO 42686 Fun Indoor Playground</t>
+  </si>
+  <si>
+    <t>LEGO City 60505 Airplane, Service Truck &amp;...</t>
+  </si>
+  <si>
+    <t>LEGO 60503 Coast Guard Helicopter</t>
+  </si>
+  <si>
+    <t>LEGO 42671 Plant Café &amp; Flower Shop</t>
+  </si>
+  <si>
+    <t>LEGO Icons 11376 Ford Model T 11376</t>
+  </si>
+  <si>
+    <t>LEGO 60504 Coast Guard Rescue Boat &amp; Helicopter</t>
+  </si>
+  <si>
     <t>LEGO 75459 Imperial Lambda-Class Shuttle</t>
   </si>
   <si>
-    <t>LEGO 42688 Horse Stable and Riding Academy</t>
-  </si>
-  <si>
-    <t>LEGO 42671 Plant Café &amp; Flower Shop</t>
-  </si>
-  <si>
-    <t>LEGO Star Wars 75453 Offworld Sandcrawler and...</t>
-  </si>
-  <si>
-    <t>LEGO 75452 BB-8 Astromech Droid</t>
-  </si>
-  <si>
-    <t>LEGO 42689 Heartlake City Friends Club House</t>
-  </si>
-  <si>
     <t>LEGO 75461 Up-Scaled Darth Vader Minifigure</t>
   </si>
   <si>
-    <t>LEGO Star Wars 75455 Boba Fett 75455</t>
-  </si>
-  <si>
     <t>LEGO 42674 Comic Book and Game Store</t>
   </si>
   <si>
+    <t>LEGO 75458 Imperial Remnant AT-RT Driver Helmet</t>
+  </si>
+  <si>
+    <t>LEGO 42685 Heartlake City Fashion Show</t>
+  </si>
+  <si>
+    <t>LEGO 42699 Beach House with Seals</t>
+  </si>
+  <si>
+    <t>LEGO Friends 42703 Mermaid Roller Coaster Ride...</t>
+  </si>
+  <si>
+    <t>LEGO Friends 42705 Cozy Fall Forest Cabin 42705</t>
+  </si>
+  <si>
     <t>LEGO Friends 42704 Heartlake City Grand Hotel...</t>
-  </si>
-  <si>
-    <t>LEGO Icons 10335 The Endurance 10335</t>
-  </si>
-  <si>
-    <t>LEGO 75458 Imperial Remnant AT-RT Driver Helmet</t>
-  </si>
-  <si>
-    <t>LEGO 60508 Police Train Heist</t>
-  </si>
-  <si>
-    <t>LEGO Star Wars 75454 Imperial Remnant AT-AT...</t>
-  </si>
-  <si>
-    <t>LEGO 42686 Fun Indoor Playground</t>
-  </si>
-  <si>
-    <t>LEGO Friends 42703 Mermaid Roller Coaster Ride...</t>
   </si>
 </sst>
 </file>
@@ -472,13 +472,13 @@
         <v>249.99</v>
       </c>
       <c r="E2">
-        <v>310.52</v>
+        <v>284.62</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="G2">
-        <v>60.52999999999997</v>
+        <v>34.63</v>
       </c>
       <c r="H2" t="s">
         <v>1</v>
@@ -491,23 +491,26 @@
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3">
-        <v>175.62</v>
-      </c>
       <c r="C3">
-        <v>125.99</v>
+        <v>55.99</v>
+      </c>
+      <c r="D3">
+        <v>81.97</v>
+      </c>
+      <c r="E3">
+        <v>69.12</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>49.63000000000001</v>
+        <v>25.98</v>
       </c>
       <c r="H3" t="s">
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -521,16 +524,16 @@
         <v>110.49</v>
       </c>
       <c r="D4">
-        <v>117.5</v>
+        <v>117.1</v>
       </c>
       <c r="E4">
-        <v>144.16</v>
+        <v>132.14</v>
       </c>
       <c r="F4">
         <v>4</v>
       </c>
       <c r="G4">
-        <v>35.70999999999999</v>
+        <v>23.68999999999998</v>
       </c>
       <c r="H4" t="s">
         <v>0</v>
@@ -543,46 +546,49 @@
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B5">
-        <v>80.55</v>
+      <c r="C5">
+        <v>71.98999999999999</v>
       </c>
       <c r="D5">
-        <v>90.47</v>
+        <v>93.68000000000001</v>
       </c>
       <c r="E5">
-        <v>110.89</v>
+        <v>78.26000000000001</v>
       </c>
       <c r="F5">
         <v>3</v>
       </c>
       <c r="G5">
-        <v>30.34</v>
+        <v>21.69000000000001</v>
       </c>
       <c r="H5" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="C6">
-        <v>149.99</v>
+      <c r="B6">
+        <v>80.55</v>
+      </c>
+      <c r="D6">
+        <v>90.16</v>
       </c>
       <c r="E6">
-        <v>177.44</v>
+        <v>101.64</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G6">
-        <v>27.44999999999999</v>
+        <v>21.09</v>
       </c>
       <c r="H6" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="s">
         <v>3</v>
@@ -593,19 +599,19 @@
         <v>14</v>
       </c>
       <c r="C7">
-        <v>55.99</v>
+        <v>47.99</v>
       </c>
       <c r="D7">
-        <v>82.25</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="E7">
-        <v>75.41</v>
+        <v>51.83</v>
       </c>
       <c r="F7">
         <v>3</v>
       </c>
       <c r="G7">
-        <v>26.26</v>
+        <v>16.41</v>
       </c>
       <c r="H7" t="s">
         <v>1</v>
@@ -618,49 +624,55 @@
       <c r="A8" t="s">
         <v>15</v>
       </c>
+      <c r="B8">
+        <v>54.61</v>
+      </c>
       <c r="C8">
-        <v>76.48999999999999</v>
+        <v>55.99</v>
+      </c>
+      <c r="D8">
+        <v>70.25</v>
       </c>
       <c r="E8">
-        <v>99.79000000000001</v>
+        <v>60.98</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G8">
-        <v>23.30000000000001</v>
+        <v>15.64</v>
       </c>
       <c r="H8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="B9">
-        <v>165.28</v>
-      </c>
       <c r="C9">
-        <v>169.99</v>
+        <v>41.99</v>
+      </c>
+      <c r="D9">
+        <v>57.37</v>
       </c>
       <c r="E9">
-        <v>188.53</v>
+        <v>51.83</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9">
-        <v>23.25</v>
+        <v>15.38</v>
       </c>
       <c r="H9" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -668,16 +680,16 @@
         <v>17</v>
       </c>
       <c r="C10">
-        <v>62.99</v>
+        <v>76.48999999999999</v>
       </c>
       <c r="E10">
-        <v>85.38</v>
+        <v>91.47</v>
       </c>
       <c r="F10">
         <v>2</v>
       </c>
       <c r="G10">
-        <v>22.38999999999999</v>
+        <v>14.98</v>
       </c>
       <c r="H10" t="s">
         <v>1</v>
@@ -690,26 +702,23 @@
       <c r="A11" t="s">
         <v>18</v>
       </c>
+      <c r="B11">
+        <v>108.45</v>
+      </c>
       <c r="C11">
-        <v>71.98999999999999</v>
-      </c>
-      <c r="D11">
-        <v>94</v>
-      </c>
-      <c r="E11">
-        <v>85.38</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>22.01000000000001</v>
+        <v>13.46000000000001</v>
       </c>
       <c r="H11" t="s">
         <v>1</v>
       </c>
       <c r="I11" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -717,45 +726,45 @@
         <v>19</v>
       </c>
       <c r="C12">
-        <v>99.98999999999999</v>
+        <v>87.98999999999999</v>
+      </c>
+      <c r="D12">
+        <v>100.7</v>
       </c>
       <c r="E12">
-        <v>121.98</v>
+        <v>95.54000000000001</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12">
-        <v>21.99000000000001</v>
+        <v>12.71000000000001</v>
       </c>
       <c r="H12" t="s">
         <v>1</v>
       </c>
       <c r="I12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>20</v>
       </c>
-      <c r="B13">
-        <v>139.45</v>
-      </c>
       <c r="C13">
-        <v>144.49</v>
+        <v>149.99</v>
       </c>
       <c r="E13">
-        <v>160.8</v>
+        <v>162.63</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>21.35000000000002</v>
+        <v>12.63999999999999</v>
       </c>
       <c r="H13" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="s">
         <v>3</v>
@@ -766,16 +775,16 @@
         <v>21</v>
       </c>
       <c r="C14">
-        <v>89.98999999999999</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="E14">
-        <v>110.89</v>
+        <v>111.81</v>
       </c>
       <c r="F14">
         <v>2</v>
       </c>
       <c r="G14">
-        <v>20.90000000000001</v>
+        <v>11.82000000000001</v>
       </c>
       <c r="H14" t="s">
         <v>1</v>
@@ -788,23 +797,20 @@
       <c r="A15" t="s">
         <v>22</v>
       </c>
-      <c r="B15">
-        <v>122.04</v>
-      </c>
       <c r="C15">
-        <v>127.49</v>
+        <v>89.98999999999999</v>
       </c>
       <c r="E15">
-        <v>141.94</v>
+        <v>101.64</v>
       </c>
       <c r="F15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G15">
-        <v>19.89999999999999</v>
+        <v>11.65000000000001</v>
       </c>
       <c r="H15" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" t="s">
         <v>3</v>
@@ -814,23 +820,23 @@
       <c r="A16" t="s">
         <v>23</v>
       </c>
-      <c r="B16">
-        <v>289.28</v>
-      </c>
       <c r="C16">
-        <v>269.99</v>
+        <v>69.98999999999999</v>
+      </c>
+      <c r="E16">
+        <v>81.31</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>19.28999999999996</v>
+        <v>11.32000000000001</v>
       </c>
       <c r="H16" t="s">
         <v>1</v>
       </c>
       <c r="I16" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -838,22 +844,25 @@
         <v>24</v>
       </c>
       <c r="C17">
-        <v>69.98999999999999</v>
+        <v>42.49</v>
+      </c>
+      <c r="D17">
+        <v>52.69</v>
       </c>
       <c r="E17">
-        <v>88.70999999999999</v>
+        <v>43.7</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17">
-        <v>18.72</v>
+        <v>10.2</v>
       </c>
       <c r="H17" t="s">
         <v>1</v>
       </c>
       <c r="I17" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -861,22 +870,25 @@
         <v>25</v>
       </c>
       <c r="C18">
-        <v>169.99</v>
+        <v>42.49</v>
+      </c>
+      <c r="D18">
+        <v>52.69</v>
       </c>
       <c r="E18">
-        <v>188.53</v>
+        <v>50.82</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G18">
-        <v>18.53999999999999</v>
+        <v>10.2</v>
       </c>
       <c r="H18" t="s">
         <v>1</v>
       </c>
       <c r="I18" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -884,19 +896,19 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>132.58</v>
+        <v>77.86</v>
       </c>
       <c r="C19">
-        <v>135.99</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="E19">
-        <v>150.82</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F19">
         <v>3</v>
       </c>
       <c r="G19">
-        <v>18.23999999999998</v>
+        <v>8.540000000000006</v>
       </c>
       <c r="H19" t="s">
         <v>0</v>
@@ -909,26 +921,26 @@
       <c r="A20" t="s">
         <v>27</v>
       </c>
+      <c r="B20">
+        <v>77.86</v>
+      </c>
       <c r="C20">
-        <v>47.99</v>
-      </c>
-      <c r="D20">
-        <v>64.62</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="E20">
-        <v>56.55</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F20">
         <v>3</v>
       </c>
       <c r="G20">
-        <v>16.63</v>
+        <v>8.540000000000006</v>
       </c>
       <c r="H20" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -936,19 +948,19 @@
         <v>28</v>
       </c>
       <c r="B21">
-        <v>77.86</v>
+        <v>122.04</v>
       </c>
       <c r="C21">
-        <v>84.98999999999999</v>
+        <v>127.49</v>
       </c>
       <c r="E21">
-        <v>94.26000000000001</v>
+        <v>130.1</v>
       </c>
       <c r="F21">
         <v>3</v>
       </c>
       <c r="G21">
-        <v>16.40000000000001</v>
+        <v>8.059999999999988</v>
       </c>
       <c r="H21" t="s">
         <v>0</v>

</xml_diff>